<commit_message>
Fixed how ParameterRetriever values are updated according to scenarios and updated tests. Now supports both rel and abs values and multiple scenarios.
</commit_message>
<xml_diff>
--- a/tests/retriever_test.xlsx
+++ b/tests/retriever_test.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="19">
   <si>
     <t>f_A</t>
   </si>
@@ -70,6 +70,12 @@
   </si>
   <si>
     <t>d3</t>
+  </si>
+  <si>
+    <t>a2</t>
+  </si>
+  <si>
+    <t>c2</t>
   </si>
 </sst>
 </file>
@@ -387,7 +393,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -469,32 +475,49 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D7" t="s">
-        <v>15</v>
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>18</v>
       </c>
       <c r="E7" t="s">
         <v>8</v>
       </c>
       <c r="F7">
-        <v>3</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
       <c r="D8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
         <v>16</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E9" t="s">
         <v>9</v>
       </c>
-      <c r="F8">
+      <c r="F9">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E9" t="s">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E10" t="s">
         <v>10</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F10" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added possibility to have columns as filters when reading data from csv
</commit_message>
<xml_diff>
--- a/tests/retriever_test.xlsx
+++ b/tests/retriever_test.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="21">
   <si>
     <t>f_A</t>
   </si>
@@ -76,6 +76,12 @@
   </si>
   <si>
     <t>c2</t>
+  </si>
+  <si>
+    <t>six</t>
+  </si>
+  <si>
+    <t>retriever_test2.csv</t>
   </si>
 </sst>
 </file>
@@ -393,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -521,6 +527,14 @@
         <v>11</v>
       </c>
     </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E11" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>